<commit_message>
chore: checkpoint current mycheck changes
</commit_message>
<xml_diff>
--- a/templates/mycheck-template.xlsx
+++ b/templates/mycheck-template.xlsx
@@ -21,14 +21,15 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IncidentIndex" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IncidentCategories" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Notifications" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Entries" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EntryLogs" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handovers" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HandoverAcks" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Incidents" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IncidentNotes" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Photos" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AuditLog" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Drafts" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Entries" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EntryLogs" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Handovers" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HandoverAcks" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Incidents" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IncidentNotes" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Photos" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AuditLog" sheetId="23" state="visible" r:id="rId23"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'_meta'!$A$1:$B$1</definedName>
@@ -45,14 +46,15 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'IncidentIndex'!$A$1:$I$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'IncidentCategories'!$A$1:$G$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Notifications'!$A$1:$H$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Entries'!$A$1:$O$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'EntryLogs'!$A$1:$P$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'Handovers'!$A$1:$I$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'HandoverAcks'!$A$1:$F$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'Incidents'!$A$1:$U$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'IncidentNotes'!$A$1:$F$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'Photos'!$A$1:$Q$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="21" hidden="1">'AuditLog'!$A$1:$N$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Drafts'!$A$1:$I$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'Entries'!$A$1:$O$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'EntryLogs'!$A$1:$P$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'Handovers'!$A$1:$I$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'HandoverAcks'!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'Incidents'!$A$1:$U$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'IncidentNotes'!$A$1:$F$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="21" hidden="1">'Photos'!$A$1:$Q$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="22" hidden="1">'AuditLog'!$A$1:$N$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -528,7 +530,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-10-18T02:36:11.099227+00:00</t>
+          <t>2026-10-18T08:37:28.123103+00:00</t>
         </is>
       </c>
     </row>
@@ -951,6 +953,79 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>shift_instance_id</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>user_id</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>shift_date</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>payload</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>client_updated_at</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>updated_at</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>version</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:I1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:O1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1054,7 +1129,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1169,7 +1244,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1242,7 +1317,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1297,7 +1372,86 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>start_time</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>end_time</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>crosses_midnight</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>sort_order</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>is_active</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>created_at</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>updated_at</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>version</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:J1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1442,86 +1596,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>start_time</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>end_time</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>crosses_midnight</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>sort_order</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>is_active</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>created_at</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>updated_at</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>version</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:J1"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1576,7 +1651,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1697,7 +1772,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>